<commit_message>
Make WINGS build manual-only and always scrape
The nightly cron could never succeed: schedule runs pass no `months`, so
the workflow skipped scraping and looked for a WINGS export in wings_data/,
which .gitignore keeps out of the repo. build_data.py then exited 1.

Drop the schedule, require `months` on dispatch, and always scrape.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_rules/model_mapping.xlsx
+++ b/model_rules/model_mapping.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -852,7 +852,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2646 LS</t>
+          <t>2646 LSDNA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2651 LS</t>
+          <t>2651 LSDNA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2653 LS</t>
+          <t>2653 LSDNA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2663 LS</t>
+          <t>2663 LSDNA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2663 LS</t>
+          <t>2663 LSDNA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2663 LS</t>
+          <t>2663 LSDNA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2663 LS</t>
+          <t>2663 LSDNA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Mismatch</t>
+          <t>Match</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Internal quotation_CG05  Arocs 2851L 6x4 C3M Tanker 2026-04_(1).docx</t>
+          <t>Internal quotation_CG04  Arocs 2851L 6x4 S5F 2026-09_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2009,27 +2009,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>4153 K</t>
+          <t>2851 L</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3253 K</t>
+          <t>2651 L</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4153 K</t>
+          <t>2851L</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>96423012</t>
+          <t>96402412</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>26A</t>
+          <t>27B</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_CG05  Arocs 2851L 6x4 C3M Tanker 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 PPC 2026-09_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>4153 K 8x4</t>
+          <t>4153 K</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 PPC 2026-09_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2150,27 +2150,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>4153 L</t>
+          <t>4153 K 8x4</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3253 L</t>
+          <t>3253 K</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4153L</t>
+          <t>4153 K</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>96403812</t>
+          <t>96423012</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>27B</t>
+          <t>26A</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02 Arocs 4153L 8x4 S5F 2026-04_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02-1 Arocs 4153L 8x4 S5F 2026-08_(1).docx</t>
+          <t>Internal quotation_CG02 Arocs 4153L 8x4 S5F 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02-2 Arocs 4153L 8x4 S5F PPC 2026-09_(1).docx</t>
+          <t>Internal quotation_CG02-1 Arocs 4153L 8x4 S5F 2026-08_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Internal quotation_CG03 Arocs 5 4153L C3M 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_CG02-2 Arocs 4153L 8x4 S5F PPC 2026-09_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2338,22 +2338,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>4153 L</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>3253 L</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>4153L</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>96403112</t>
+          <t>96403812</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Internal quotation_E05 Arocs 4440 C3H-S 8x4 Classic Euro5 FA9t- UAE 2026-06_(1).docx</t>
+          <t>Internal quotation_CG03 Arocs 5 4153L C3M 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2385,40 +2385,87 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>4440</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>4440</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>4440</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>96403112</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>27B</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>PTO</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Internal quotation_E05 Arocs 4440 C3H-S 8x4 Classic Euro5 FA9t- UAE 2026-06_(1).docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Arocs</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>4453 K</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>4153 K</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>4453K</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>96423112</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>26A</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>PTO</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>PTO</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>Internal quotation_DP02  Arocs 4453K 8x4 Hub 2026-05_(1).docx</t>
         </is>

</xml_diff>

<commit_message>
Update model mapping, category, and data.json
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_rules/model_mapping.xlsx
+++ b/model_rules/model_mapping.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Match</t>
+          <t>Mismatch</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Internal quotation_CG04  Arocs 2851L 6x4 S5F 2026-09_(1).docx</t>
+          <t>Internal quotation_CG05  Arocs 2851L 6x4 C3M Tanker 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2009,27 +2009,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2851 L</t>
+          <t>4153 K</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2651 L</t>
+          <t>3253 K</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2851L</t>
+          <t>4153 K</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>96402412</t>
+          <t>96423012</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>27B</t>
+          <t>26A</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Internal quotation_CG05  Arocs 2851L 6x4 C3M Tanker 2026-04_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 PPC 2026-09_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2103,19 +2103,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>4153 K 8x4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3253 K</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>4153 K</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>3253 K</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>4153 K</t>
-        </is>
-      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>96423012</t>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 PPC 2026-09_(1).docx</t>
+          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2150,27 +2150,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>4153 K 8x4</t>
+          <t>4153 L</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3253 K</t>
+          <t>3253 L</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4153 K</t>
+          <t>4153L</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>96423012</t>
+          <t>96403812</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>26A</t>
+          <t>27B</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Internal quotation_DP01 Arocs 4153 K 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_CG02 Arocs 4153L 8x4 S5F 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02 Arocs 4153L 8x4 S5F 2026-04_(1).docx</t>
+          <t>Internal quotation_CG02-1 Arocs 4153L 8x4 S5F 2026-08_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02-1 Arocs 4153L 8x4 S5F 2026-08_(1).docx</t>
+          <t>Internal quotation_CG02-2 Arocs 4153L 8x4 S5F PPC 2026-09_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Internal quotation_CG02-2 Arocs 4153L 8x4 S5F PPC 2026-09_(1).docx</t>
+          <t>Internal quotation_CG03 Arocs 5 4153L C3M 8x4 2026-04_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2338,22 +2338,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4153 L</t>
+          <t>4440</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3253 L</t>
+          <t>4440</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4153L</t>
+          <t>4440</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>96403812</t>
+          <t>96403112</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Internal quotation_CG03 Arocs 5 4153L C3M 8x4 2026-04_(1).docx</t>
+          <t>Internal quotation_E05 Arocs 4440 C3H-S 8x4 Classic Euro5 FA9t- UAE 2026-06_(1).docx</t>
         </is>
       </c>
     </row>
@@ -2385,27 +2385,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>4453 K</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>4153 K</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>4440</t>
+          <t>4453K</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>96403112</t>
+          <t>96423112</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>27B</t>
+          <t>26A</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2419,53 +2419,6 @@
         </is>
       </c>
       <c r="I46" t="inlineStr">
-        <is>
-          <t>Internal quotation_E05 Arocs 4440 C3H-S 8x4 Classic Euro5 FA9t- UAE 2026-06_(1).docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Arocs</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>4453 K</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>4153 K</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>4453K</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>96423112</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>26A</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>PTO</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
         <is>
           <t>Internal quotation_DP02  Arocs 4453K 8x4 Hub 2026-05_(1).docx</t>
         </is>

</xml_diff>